<commit_message>
#61 R71,R72 Added in Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Solenoid-Board-v2.0/BOM/Client-Solenoid-Board-v2.0.xlsx
+++ b/Design Files/Solenoid-Board-v2.0/BOM/Client-Solenoid-Board-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="284">
   <si>
     <t>#</t>
   </si>
@@ -859,6 +859,18 @@
   </si>
   <si>
     <t xml:space="preserve">Solenoid </t>
+  </si>
+  <si>
+    <t>R71, R72</t>
+  </si>
+  <si>
+    <t>RES 560 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07560RL</t>
+  </si>
+  <si>
+    <t>560R</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1374,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1375,6 +1387,8 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1458,7 +1472,7 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B55" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B56" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -2868,412 +2882,443 @@
         <v>46</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>69</v>
+        <v>280</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>124</v>
+        <v>281</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>264</v>
+        <v>160</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>162</v>
+        <v>282</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="J48" s="7">
         <v>2</v>
       </c>
       <c r="K48" s="7"/>
     </row>
-    <row r="49" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B49) - ROW($B$2)</f>
         <v>47</v>
       </c>
-      <c r="C49" s="13" t="s">
+      <c r="C49" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>125</v>
+      <c r="D49" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="G49" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>238</v>
+      <c r="G49" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J49" s="9">
-        <v>1</v>
-      </c>
-      <c r="K49" s="9"/>
-    </row>
-    <row r="50" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J49" s="7">
+        <v>2</v>
+      </c>
+      <c r="K49" s="7"/>
+    </row>
+    <row r="50" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
-        <f>ROW(B50) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C50" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>126</v>
+      <c r="C50" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G50" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>239</v>
+        <v>264</v>
+      </c>
+      <c r="G50" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H50" s="9" t="s">
+        <v>238</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J50" s="7">
-        <v>1</v>
-      </c>
-      <c r="K50" s="7"/>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J50" s="9">
+        <v>1</v>
+      </c>
+      <c r="K50" s="9"/>
+    </row>
+    <row r="51" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B51) - ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="C51" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D51" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>7</v>
+      <c r="D51" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>239</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J51" s="9">
-        <v>1</v>
-      </c>
-      <c r="K51" s="9"/>
+      <c r="J51" s="7">
+        <v>1</v>
+      </c>
+      <c r="K51" s="7"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
-        <f>ROW(B52) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D52" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="H52" s="7" t="s">
-        <v>227</v>
+      <c r="D52" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>7</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J52" s="7">
-        <v>1</v>
-      </c>
-      <c r="K52" s="7"/>
+      <c r="J52" s="9">
+        <v>1</v>
+      </c>
+      <c r="K52" s="9"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B53) - ROW($B$2)</f>
         <v>51</v>
       </c>
-      <c r="C53" s="13" t="s">
+      <c r="C53" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>239</v>
+      <c r="D53" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>227</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J53" s="9">
-        <v>1</v>
-      </c>
-      <c r="K53" s="9"/>
+      <c r="J53" s="7">
+        <v>1</v>
+      </c>
+      <c r="K53" s="7"/>
     </row>
     <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
-        <f>ROW(B54) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C54" s="12" t="s">
+      <c r="C54" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D54" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E54" s="8" t="s">
+      <c r="D54" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E54" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="F54" s="7" t="s">
+      <c r="F54" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="G54" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="H54" s="7" t="s">
+      <c r="G54" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H54" s="9" t="s">
         <v>239</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J54" s="7">
-        <v>1</v>
-      </c>
-      <c r="K54" s="7"/>
+      <c r="J54" s="9">
+        <v>1</v>
+      </c>
+      <c r="K54" s="9"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B55) - ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="13" t="s">
+      <c r="C55" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D55" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="G55" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>227</v>
+      <c r="D55" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>239</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J55" s="9">
-        <v>1</v>
-      </c>
-      <c r="K55" s="9"/>
-    </row>
-    <row r="56" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J55" s="7">
+        <v>1</v>
+      </c>
+      <c r="K55" s="7"/>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f>ROW(B56) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D56" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>239</v>
+      <c r="D56" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="G56" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>227</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J56" s="7">
-        <v>4</v>
-      </c>
-      <c r="K56" s="7"/>
+      <c r="J56" s="9">
+        <v>1</v>
+      </c>
+      <c r="K56" s="9"/>
     </row>
     <row r="57" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="11">
-        <f t="shared" ref="B57" si="1">ROW(B57) - ROW($B$2)</f>
+        <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="G57" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="I57" s="10" t="s">
-        <v>263</v>
-      </c>
-      <c r="J57" s="9">
-        <v>1</v>
-      </c>
-      <c r="K57" s="9"/>
+      <c r="C57" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="I57" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="J57" s="7">
+        <v>4</v>
+      </c>
+      <c r="K57" s="7"/>
     </row>
     <row r="58" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B58" s="11">
-        <f>ROW(B58) - ROW($B$2)</f>
+        <f t="shared" ref="B58" si="1">ROW(B58) - ROW($B$2)</f>
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>269</v>
+      <c r="D58" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>278</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="G58" s="8" t="s">
-        <v>270</v>
-      </c>
-      <c r="H58" s="7" t="s">
-        <v>271</v>
+      <c r="G58" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>229</v>
       </c>
       <c r="I58" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="J58" s="7">
-        <v>2</v>
-      </c>
-      <c r="K58" s="7"/>
-    </row>
-    <row r="59" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J58" s="9">
+        <v>1</v>
+      </c>
+      <c r="K58" s="9"/>
+    </row>
+    <row r="59" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="11">
-        <f t="shared" ref="B59" si="2">ROW(B59) - ROW($B$2)</f>
+        <f>ROW(B59) - ROW($B$2)</f>
         <v>57</v>
       </c>
       <c r="C59" s="13" t="s">
         <v>266</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>264</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="J59" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="K59" s="14" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>271</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="J59" s="7">
+        <v>2</v>
+      </c>
+      <c r="K59" s="7"/>
+    </row>
+    <row r="60" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B60" s="11">
-        <f>ROW(B60) - ROW($B$2)</f>
+        <f t="shared" ref="B60" si="2">ROW(B60) - ROW($B$2)</f>
         <v>58</v>
       </c>
       <c r="C60" s="13" t="s">
         <v>266</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>264</v>
       </c>
       <c r="G60" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="J60" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="K60" s="14" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="11">
+        <f>ROW(B61) - ROW($B$2)</f>
+        <v>59</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="G61" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="H60" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="I60" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="J60" s="7">
-        <v>1</v>
-      </c>
-      <c r="K60" s="14" t="s">
+      <c r="H61" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="J61" s="7">
+        <v>1</v>
+      </c>
+      <c r="K61" s="14" t="s">
         <v>276</v>
       </c>
     </row>

</xml_diff>